<commit_message>
cretae folder - DeviceIdentifierLibrary.ManualTest
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/SolutionOverview.xlsx
+++ b/1.training_model/supplementary/SolutionOverview.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\slide_presentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{870A895B-6D18-435D-8A2C-10E07F21E849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86F283B-AB23-4202-AFB0-A58D6BB5C3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F786F84-E58A-4E84-A5D5-55259F2E6D26}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="63">
   <si>
     <t>Model</t>
   </si>
@@ -106,6 +106,114 @@
   </si>
   <si>
     <t>Handles Python execution logic</t>
+  </si>
+  <si>
+    <t>Access Modifier</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Program</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>Main Class</t>
+  </si>
+  <si>
+    <t>Entry point of the application (contains Main method)</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>_baseDir</t>
+  </si>
+  <si>
+    <t>private</t>
+  </si>
+  <si>
+    <t>static field</t>
+  </si>
+  <si>
+    <t>Stores base directory path</t>
+  </si>
+  <si>
+    <t>_projectDir</t>
+  </si>
+  <si>
+    <t>Stores project directory path</t>
+  </si>
+  <si>
+    <t>_serviceDir</t>
+  </si>
+  <si>
+    <t>Stores service directory path</t>
+  </si>
+  <si>
+    <t>PYTHON_EXE</t>
+  </si>
+  <si>
+    <t>Python executable path</t>
+  </si>
+  <si>
+    <t>SCRIPT_TYPE</t>
+  </si>
+  <si>
+    <t>Path to predict_equipment.py</t>
+  </si>
+  <si>
+    <t>SCRIPT_PIPELINE</t>
+  </si>
+  <si>
+    <t>Path to predict_sectioncluster.py</t>
+  </si>
+  <si>
+    <t>PROJECT_JSON</t>
+  </si>
+  <si>
+    <t>Path to input JSON file</t>
+  </si>
+  <si>
+    <t>_jsonOpts</t>
+  </si>
+  <si>
+    <t>JSON serializer options</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Main</t>
+  </si>
+  <si>
+    <t>static method</t>
+  </si>
+  <si>
+    <t>Main execution flow (calls prediction steps)</t>
+  </si>
+  <si>
+    <t>PrintDeviceTypeTable</t>
+  </si>
+  <si>
+    <t>Prints device type results</t>
+  </si>
+  <si>
+    <t>PrintSectionTable</t>
+  </si>
+  <si>
+    <t>Prints section results</t>
+  </si>
+  <si>
+    <t>PrintClusterTable</t>
+  </si>
+  <si>
+    <t>Prints cluster results</t>
   </si>
 </sst>
 </file>
@@ -504,16 +612,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874B85AB-2F67-4FFD-B7D4-6742BD17433A}">
-  <dimension ref="B2:E10"/>
+  <dimension ref="B2:F29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
@@ -527,7 +635,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
@@ -541,7 +649,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -555,7 +663,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
@@ -569,7 +677,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -583,7 +691,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -597,7 +705,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
@@ -611,7 +719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
@@ -625,7 +733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>24</v>
       </c>
@@ -637,6 +745,244 @@
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" t="s">
+        <v>55</v>
+      </c>
+      <c r="F26" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" t="s">
+        <v>36</v>
+      </c>
+      <c r="E27" t="s">
+        <v>55</v>
+      </c>
+      <c r="F27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28" t="s">
+        <v>55</v>
+      </c>
+      <c r="F28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" t="s">
+        <v>55</v>
+      </c>
+      <c r="F29" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removal folder - ManualTest
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/SolutionOverview.xlsx
+++ b/1.training_model/supplementary/SolutionOverview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86F283B-AB23-4202-AFB0-A58D6BB5C3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC02B04-1BDD-4C9A-A9C9-0CC83DD46807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F786F84-E58A-4E84-A5D5-55259F2E6D26}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="70">
   <si>
     <t>Model</t>
   </si>
@@ -214,6 +214,27 @@
   </si>
   <si>
     <t>Prints cluster results</t>
+  </si>
+  <si>
+    <t>DevicePredictRequest</t>
+  </si>
+  <si>
+    <t>ManualAssignment</t>
+  </si>
+  <si>
+    <t>UserManualAssignRequest</t>
+  </si>
+  <si>
+    <t>PipelinePredictRequest</t>
+  </si>
+  <si>
+    <t>PipelineRecord</t>
+  </si>
+  <si>
+    <t>DeviceTypeResult</t>
+  </si>
+  <si>
+    <t>PipelineResult</t>
   </si>
 </sst>
 </file>
@@ -237,12 +258,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -272,12 +299,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,16 +644,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874B85AB-2F67-4FFD-B7D4-6742BD17433A}">
-  <dimension ref="B2:F29"/>
+  <dimension ref="B2:G34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
@@ -634,8 +667,11 @@
       <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F2" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
@@ -649,7 +685,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -663,7 +699,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
@@ -677,7 +713,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -691,7 +727,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -705,7 +741,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
@@ -718,152 +754,185 @@
       <c r="E8" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="1" t="s">
+      <c r="F13" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>2</v>
-      </c>
-      <c r="D16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" t="s">
-        <v>28</v>
-      </c>
-      <c r="F16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="F15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" t="s">
         <v>31</v>
-      </c>
-      <c r="E17" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" t="s">
-        <v>37</v>
-      </c>
-      <c r="F20" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E21" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F21" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" t="s">
-        <v>36</v>
+        <v>30</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F22" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.35">
@@ -871,16 +940,16 @@
         <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E23" t="s">
         <v>37</v>
       </c>
       <c r="F23" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.35">
@@ -888,16 +957,16 @@
         <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E24" t="s">
         <v>37</v>
       </c>
       <c r="F24" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.35">
@@ -905,83 +974,168 @@
         <v>34</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E25" t="s">
         <v>37</v>
       </c>
       <c r="F25" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="C26" t="s">
-        <v>54</v>
-      </c>
-      <c r="D26" t="s">
-        <v>31</v>
+        <v>43</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="E26" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="F26" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E27" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="F27" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D28" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E28" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" t="s">
+        <v>37</v>
+      </c>
+      <c r="F30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B31" t="s">
         <v>53</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C31" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31" t="s">
+        <v>55</v>
+      </c>
+      <c r="F31" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C32" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" t="s">
+        <v>55</v>
+      </c>
+      <c r="F32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" t="s">
+        <v>55</v>
+      </c>
+      <c r="F33" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" t="s">
         <v>61</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D34" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E34" t="s">
         <v>55</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F34" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add - ManualTest folder
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/SolutionOverview.xlsx
+++ b/1.training_model/supplementary/SolutionOverview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC02B04-1BDD-4C9A-A9C9-0CC83DD46807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53745B5C-B721-43D5-BB6F-A6001D83081D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F786F84-E58A-4E84-A5D5-55259F2E6D26}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0F786F84-E58A-4E84-A5D5-55259F2E6D26}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="91">
   <si>
     <t>Model</t>
   </si>
@@ -235,6 +235,69 @@
   </si>
   <si>
     <t>PipelineResult</t>
+  </si>
+  <si>
+    <t>FOLDER</t>
+  </si>
+  <si>
+    <t>ModelRequest</t>
+  </si>
+  <si>
+    <t>DevicePredictRequest.cs</t>
+  </si>
+  <si>
+    <t>updated on 11/06/2026</t>
+  </si>
+  <si>
+    <t>PipelinePredictRequest.cs</t>
+  </si>
+  <si>
+    <t>ManualAssignment.cs</t>
+  </si>
+  <si>
+    <t>PipelineRecord.cs</t>
+  </si>
+  <si>
+    <t>UserManualAssignRequest.cs</t>
+  </si>
+  <si>
+    <t>ModelResult</t>
+  </si>
+  <si>
+    <t>DeviceTypeResult.cs</t>
+  </si>
+  <si>
+    <t>PipelineResult.cs</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>SCRIPT</t>
+  </si>
+  <si>
+    <t>CLASS</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>FUNCTION OF CLASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hold a string format </t>
+  </si>
+  <si>
+    <t>(customer, data_id, manual_check, confidence, reason)</t>
+  </si>
+  <si>
+    <t>FORMAT</t>
+  </si>
+  <si>
+    <t>(DEVICE_ID, CUSTOMER, PROJECT, PREDICTED_SECTION, SECTION_CONFIDENCE, PREDICTED_CLUSTER, CLUSTER_CONFIDENCE, REJECTION_REASON, FORMAT_WARNING)</t>
+  </si>
+  <si>
+    <t>EXIST</t>
   </si>
 </sst>
 </file>
@@ -258,7 +321,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -271,8 +334,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -295,21 +364,144 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -644,17 +836,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874B85AB-2F67-4FFD-B7D4-6742BD17433A}">
-  <dimension ref="B2:G34"/>
+  <dimension ref="A2:H50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="66" customWidth="1"/>
+    <col min="8" max="8" width="6.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
@@ -667,11 +862,12 @@
       <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
@@ -685,7 +881,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -699,7 +895,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
@@ -713,7 +909,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -727,7 +923,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -741,7 +937,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
@@ -757,11 +953,11 @@
       <c r="F8" t="s">
         <v>63</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
@@ -777,11 +973,11 @@
       <c r="F9" t="s">
         <v>64</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
@@ -797,11 +993,11 @@
       <c r="F10" t="s">
         <v>65</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>0</v>
       </c>
@@ -817,11 +1013,11 @@
       <c r="F11" t="s">
         <v>66</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
@@ -837,11 +1033,11 @@
       <c r="F12" t="s">
         <v>67</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
@@ -857,11 +1053,11 @@
       <c r="F13" t="s">
         <v>68</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
@@ -877,11 +1073,11 @@
       <c r="F14" t="s">
         <v>69</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
@@ -891,251 +1087,400 @@
       <c r="D15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F15" t="s">
         <v>25</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
+    <row r="19" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C20" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C21" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C22" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C23" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C24" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C25" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C26" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="G26" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="H26" s="16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C27" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F27" s="14"/>
+      <c r="G27" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="H27" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C28" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="19"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B37" t="s">
         <v>9</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C37" t="s">
         <v>2</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D37" t="s">
         <v>27</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E37" t="s">
         <v>28</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F37" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B38" t="s">
         <v>29</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C38" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D38" t="s">
         <v>31</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E38" t="s">
         <v>32</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F38" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B39" t="s">
         <v>34</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C39" t="s">
         <v>35</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D39" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E39" t="s">
         <v>37</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F39" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B40" t="s">
         <v>34</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C40" t="s">
         <v>39</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D40" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E40" t="s">
         <v>37</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F40" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B41" t="s">
         <v>34</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C41" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D41" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E41" t="s">
         <v>37</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F41" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B42" t="s">
         <v>34</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C42" t="s">
         <v>43</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D42" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E42" t="s">
         <v>37</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F42" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B27" t="s">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B43" t="s">
         <v>34</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C43" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D43" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E43" t="s">
         <v>37</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F43" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B28" t="s">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B44" t="s">
         <v>34</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C44" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D44" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E44" t="s">
         <v>37</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F44" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B29" t="s">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B45" t="s">
         <v>34</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C45" t="s">
         <v>49</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D45" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E45" t="s">
         <v>37</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F45" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B30" t="s">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B46" t="s">
         <v>34</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C46" t="s">
         <v>51</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D46" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E46" t="s">
         <v>37</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F46" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B31" t="s">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B47" t="s">
         <v>53</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C47" t="s">
         <v>54</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D47" t="s">
         <v>31</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E47" t="s">
         <v>55</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F47" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B32" t="s">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B48" t="s">
         <v>53</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C48" t="s">
         <v>57</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D48" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E48" t="s">
         <v>55</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F48" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B33" t="s">
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B49" t="s">
         <v>53</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C49" t="s">
         <v>59</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D49" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E49" t="s">
         <v>55</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F49" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B34" t="s">
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
         <v>53</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C50" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D50" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E50" t="s">
         <v>55</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F50" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update scirpt - Program.cs
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/SolutionOverview.xlsx
+++ b/1.training_model/supplementary/SolutionOverview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{968CCD4C-68AF-479F-A5A6-39F31AC43DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D832EC8C-BEDB-4A38-A169-06326A1D0246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F786F84-E58A-4E84-A5D5-55259F2E6D26}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="116">
   <si>
     <t>Model</t>
   </si>
@@ -352,13 +352,72 @@
   </si>
   <si>
     <t>contain all the pkl file</t>
+  </si>
+  <si>
+    <t>...\DeviceCluster\DeviceIdentifierLibrary\Services</t>
+  </si>
+  <si>
+    <t>Convert SQL -&gt; JSON</t>
+  </si>
+  <si>
+    <t>import_equipment</t>
+  </si>
+  <si>
+    <t>LIST OF THE FILE INISDE predict_equipment.py</t>
+  </si>
+  <si>
+    <r>
+      <t>project_code</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>customer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>equipment_list[{data_id, equipment}]</t>
+    </r>
+  </si>
+  <si>
+    <t>user_manual_assign</t>
+  </si>
+  <si>
+    <t>project_code, customer, assignments[{data_id, equipment}]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,6 +432,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="6">
@@ -407,7 +471,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -559,11 +623,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -598,35 +673,49 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -961,8 +1050,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874B85AB-2F67-4FFD-B7D4-6742BD17433A}">
-  <dimension ref="A2:H56"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A2:H57"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
@@ -974,7 +1063,7 @@
     <col min="8" max="8" width="6.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8">
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
@@ -992,7 +1081,7 @@
       </c>
       <c r="G2" s="13"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8">
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1006,7 +1095,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8">
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1020,7 +1109,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8">
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1034,7 +1123,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1048,7 +1137,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8">
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1062,7 +1151,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8">
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
@@ -1082,7 +1171,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8">
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
@@ -1102,7 +1191,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8">
       <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1122,7 +1211,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8">
       <c r="B11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1142,7 +1231,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8">
       <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
@@ -1162,7 +1251,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8">
       <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
@@ -1182,7 +1271,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8">
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1291,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8">
       <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
@@ -1222,12 +1311,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" ht="15" thickBot="1">
       <c r="A17" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" ht="15" thickBot="1">
       <c r="C18" s="9" t="s">
         <v>70</v>
       </c>
@@ -1247,7 +1336,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8">
       <c r="C19" s="7" t="s">
         <v>71</v>
       </c>
@@ -1265,7 +1354,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8">
       <c r="C20" s="7" t="s">
         <v>71</v>
       </c>
@@ -1281,7 +1370,7 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8">
       <c r="C21" s="7" t="s">
         <v>71</v>
       </c>
@@ -1297,7 +1386,7 @@
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8">
       <c r="C22" s="7" t="s">
         <v>71</v>
       </c>
@@ -1313,7 +1402,7 @@
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
     </row>
-    <row r="23" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:8" ht="15" thickBot="1">
       <c r="C23" s="7" t="s">
         <v>71</v>
       </c>
@@ -1329,7 +1418,7 @@
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8">
       <c r="C24" s="11" t="s">
         <v>78</v>
       </c>
@@ -1347,7 +1436,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:8" ht="44" thickBot="1">
       <c r="C25" s="14" t="s">
         <v>78</v>
       </c>
@@ -1365,7 +1454,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8">
       <c r="C26" s="11" t="s">
         <v>81</v>
       </c>
@@ -1379,7 +1468,7 @@
       <c r="G26" s="11"/>
       <c r="H26" s="12"/>
     </row>
-    <row r="27" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:8" ht="15" thickBot="1">
       <c r="C27" s="8" t="s">
         <v>81</v>
       </c>
@@ -1395,148 +1484,171 @@
       </c>
       <c r="H27" s="6"/>
     </row>
-    <row r="28" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="29" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C29" s="28" t="s">
+    <row r="28" spans="1:8" ht="15" thickBot="1"/>
+    <row r="29" spans="1:8" ht="15" thickBot="1">
+      <c r="C29" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="29" t="s">
+      <c r="D29" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="E29" s="30"/>
-      <c r="F29" s="28" t="s">
+      <c r="E29" s="28"/>
+      <c r="F29" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="G29" s="28" t="s">
+      <c r="G29" s="22" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="C30" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="E30" s="21"/>
-      <c r="F30" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="G30" s="17"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8">
+      <c r="C30" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="E30" s="33"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="31" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="C31" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="E31" s="21"/>
-      <c r="F31" s="26" t="s">
+      <c r="E31" s="24"/>
+      <c r="F31" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G31" s="17"/>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="C32" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E32" s="24"/>
+      <c r="F32" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="G31" s="17" t="s">
+      <c r="G32" s="17" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="C32" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="E32" s="23"/>
-      <c r="F32" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="G32" s="18"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:7">
       <c r="C33" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D33" s="22" t="s">
+      <c r="D33" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="23"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="G33" s="18"/>
+    </row>
+    <row r="34" spans="2:7">
+      <c r="C34" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" s="26"/>
+      <c r="F34" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="G33" s="18"/>
-    </row>
-    <row r="34" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C34" s="19" t="s">
+      <c r="G34" s="18"/>
+    </row>
+    <row r="35" spans="2:7" ht="15" thickBot="1">
+      <c r="C35" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="24" t="s">
+      <c r="D35" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="25"/>
-      <c r="F34" s="27" t="s">
+      <c r="E35" s="30"/>
+      <c r="F35" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="G34" s="19" t="s">
+      <c r="G35" s="19" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:7">
+      <c r="C37" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="D37" s="35"/>
+    </row>
+    <row r="38" spans="2:7">
+      <c r="C38" t="s">
+        <v>111</v>
+      </c>
+      <c r="D38" s="36" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7">
+      <c r="C39" t="s">
+        <v>114</v>
+      </c>
+      <c r="D39" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7">
       <c r="B43" t="s">
         <v>9</v>
       </c>
-      <c r="C43" t="s">
-        <v>2</v>
-      </c>
-      <c r="D43" t="s">
-        <v>27</v>
-      </c>
-      <c r="E43" t="s">
-        <v>28</v>
-      </c>
-      <c r="F43" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="2:7">
       <c r="B44" t="s">
         <v>29</v>
       </c>
       <c r="C44" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D44" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E44" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F44" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7">
       <c r="B45" t="s">
         <v>34</v>
       </c>
       <c r="C45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
+      </c>
+      <c r="D45" t="s">
+        <v>31</v>
       </c>
       <c r="E45" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F45" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7">
       <c r="B46" t="s">
         <v>34</v>
       </c>
       <c r="C46" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>36</v>
@@ -1545,15 +1657,15 @@
         <v>37</v>
       </c>
       <c r="F46" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7">
       <c r="B47" t="s">
         <v>34</v>
       </c>
       <c r="C47" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>36</v>
@@ -1562,15 +1674,15 @@
         <v>37</v>
       </c>
       <c r="F47" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7">
       <c r="B48" t="s">
         <v>34</v>
       </c>
       <c r="C48" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>36</v>
@@ -1579,15 +1691,15 @@
         <v>37</v>
       </c>
       <c r="F48" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6">
       <c r="B49" t="s">
         <v>34</v>
       </c>
       <c r="C49" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>36</v>
@@ -1596,15 +1708,15 @@
         <v>37</v>
       </c>
       <c r="F49" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6">
       <c r="B50" t="s">
         <v>34</v>
       </c>
       <c r="C50" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>36</v>
@@ -1613,15 +1725,15 @@
         <v>37</v>
       </c>
       <c r="F50" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6">
       <c r="B51" t="s">
         <v>34</v>
       </c>
       <c r="C51" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>36</v>
@@ -1630,15 +1742,15 @@
         <v>37</v>
       </c>
       <c r="F51" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6">
       <c r="B52" t="s">
         <v>34</v>
       </c>
       <c r="C52" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>36</v>
@@ -1647,49 +1759,49 @@
         <v>37</v>
       </c>
       <c r="F52" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6">
       <c r="B53" t="s">
         <v>53</v>
       </c>
       <c r="C53" t="s">
-        <v>54</v>
-      </c>
-      <c r="D53" t="s">
-        <v>31</v>
+        <v>51</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="E53" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="F53" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6">
       <c r="B54" t="s">
         <v>53</v>
       </c>
       <c r="C54" t="s">
-        <v>57</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>36</v>
+        <v>54</v>
+      </c>
+      <c r="D54" t="s">
+        <v>31</v>
       </c>
       <c r="E54" t="s">
         <v>55</v>
       </c>
       <c r="F54" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6">
       <c r="B55" t="s">
         <v>53</v>
       </c>
       <c r="C55" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>36</v>
@@ -1698,15 +1810,15 @@
         <v>55</v>
       </c>
       <c r="F55" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6">
       <c r="B56" t="s">
         <v>53</v>
       </c>
       <c r="C56" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>36</v>
@@ -1715,16 +1827,32 @@
         <v>55</v>
       </c>
       <c r="F56" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6">
+      <c r="C57" t="s">
+        <v>61</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E57" t="s">
+        <v>55</v>
+      </c>
+      <c r="F57" t="s">
         <v>62</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="D35:E35"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C37:D37"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D32:E32"/>
     <mergeCell ref="D34:E34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>